<commit_message>
Completed the cardinality based partitioning.
</commit_message>
<xml_diff>
--- a/Experiments data/Cardinality Skewness/Skewness_4elt_Graph.xlsx
+++ b/Experiments data/Cardinality Skewness/Skewness_4elt_Graph.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengw\OneDrive\Documents\GitHub\SISR Script\Experiments data\Cardinality Skewness\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengw\OneDrive\Documents\GitHub\KaMinPar_Java\Experiments data\Cardinality Skewness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDCEE417-4718-4047-93CE-B76D817ED9A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC0D96E-ADDF-40AF-9F71-13138B00D9DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Edge Cuts" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="38">
   <si>
     <t>KaHIP</t>
   </si>
@@ -138,6 +138,18 @@
   </si>
   <si>
     <t>Deep Multilevel, ε= 0</t>
+  </si>
+  <si>
+    <t>Deep Multilevel, ε =780</t>
+  </si>
+  <si>
+    <t>Deep Multilevel, ε =100</t>
+  </si>
+  <si>
+    <t>Deep NUGP, ε =780</t>
+  </si>
+  <si>
+    <t>Deep NUGP, ε= 0</t>
   </si>
 </sst>
 </file>
@@ -324,6 +336,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -345,7 +358,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,19 +712,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3773.6</c:v>
+                  <c:v>436.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2258</c:v>
+                  <c:v>458.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>515.6</c:v>
+                  <c:v>427.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2922.2</c:v>
+                  <c:v>414.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2000.6</c:v>
+                  <c:v>405</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -733,7 +745,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε = 5</c:v>
+                  <c:v>Deep Multilevel, ε =780</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -799,19 +811,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1717.4</c:v>
+                  <c:v>375.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1157.4000000000001</c:v>
+                  <c:v>388.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>379.8</c:v>
+                  <c:v>370.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1909.8</c:v>
+                  <c:v>390</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1030</c:v>
+                  <c:v>303.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1774,7 +1786,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε= 0</c:v>
+                  <c:v>Deep NUGP, ε= 0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1834,19 +1846,19 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-9.9570267131242733</c:v>
+                  <c:v>-0.26771196283391419</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-5.5792540792540795</c:v>
+                  <c:v>-0.33508158508158509</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.49449275362318845</c:v>
+                  <c:v>-0.23826086956521736</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-7.5195335276967921</c:v>
+                  <c:v>-0.20874635568513125</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-4.8224679860302677</c:v>
+                  <c:v>-0.17869615832363206</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1867,7 +1879,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε = 5</c:v>
+                  <c:v>Deep NUGP, ε =780</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1927,19 +1939,19 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-3.9866434378629503</c:v>
+                  <c:v>-8.9430894308943132E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-2.3723776223776225</c:v>
+                  <c:v>-0.13228438228438238</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.10086956521739134</c:v>
+                  <c:v>-7.4202898550724705E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.5679300291545184</c:v>
+                  <c:v>-0.13702623906705538</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.9976717112922</c:v>
+                  <c:v>0.11757857974388833</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2123,7 +2135,7 @@
                   <a:rPr lang="en-US" sz="1800" b="0" i="0" baseline="0">
                     <a:effectLst/>
                   </a:rPr>
-                  <a:t>Percentage of Decline</a:t>
+                  <a:t>Percentage of Improvement</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US">
                   <a:effectLst/>
@@ -2559,7 +2571,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε= 0</c:v>
+                  <c:v>Deep NUGP, ε= 0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2625,19 +2637,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>5.6525999999999996</c:v>
+                  <c:v>3.1916000000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.6878000000000002</c:v>
+                  <c:v>3.0064000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6707999999999998</c:v>
+                  <c:v>3.0417999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.1120000000000001</c:v>
+                  <c:v>3.1024000000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0469999999999997</c:v>
+                  <c:v>3.9652000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2658,7 +2670,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε = 5</c:v>
+                  <c:v>Deep NUGP, ε =780</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2724,16 +2736,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.5792000000000002</c:v>
+                  <c:v>3.1394000000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2038000000000002</c:v>
+                  <c:v>3.2231999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.0680000000000001</c:v>
+                  <c:v>2.9817999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.3628</c:v>
+                  <c:v>3.0024000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>3.1444000000000001</c:v>
@@ -3907,7 +3919,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε = 5</c:v>
+                  <c:v>Deep Multilevel, ε =780</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3967,10 +3979,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.331722E-2</c:v>
+                  <c:v>0.157052</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2369800000000002E-2</c:v>
+                  <c:v>8.8782E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3.1933599999999999E-2</c:v>
@@ -4654,7 +4666,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε= 0</c:v>
+                  <c:v>Deep NUGP, ε= 0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4747,7 +4759,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Deep Multilevel, ε = 5</c:v>
+                  <c:v>Deep NUGP, ε =780</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4807,16 +4819,16 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.3126000000000001E-2</c:v>
+                  <c:v>0.10606</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4644000000000003E-2</c:v>
+                  <c:v>7.8972000000000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.1916E-2</c:v>
+                  <c:v>8.5916000000000006E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.3731999999999996E-2</c:v>
+                  <c:v>9.3916000000000013E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1.9438E-2</c:v>
@@ -10341,26 +10353,26 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
@@ -10386,7 +10398,7 @@
         <v>25</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -10412,10 +10424,10 @@
         <v>341</v>
       </c>
       <c r="H5">
-        <v>2888</v>
+        <v>410</v>
       </c>
       <c r="I5">
-        <v>1337</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -10441,10 +10453,10 @@
         <v>357</v>
       </c>
       <c r="H6">
-        <v>2061</v>
+        <v>460</v>
       </c>
       <c r="I6">
-        <v>1794</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -10470,10 +10482,10 @@
         <v>341</v>
       </c>
       <c r="H7">
-        <v>5373</v>
+        <v>474</v>
       </c>
       <c r="I7">
-        <v>1608</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -10499,10 +10511,10 @@
         <v>341</v>
       </c>
       <c r="H8">
-        <v>3503</v>
+        <v>453</v>
       </c>
       <c r="I8">
-        <v>2051</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -10528,10 +10540,10 @@
         <v>342</v>
       </c>
       <c r="H9">
-        <v>5043</v>
+        <v>386</v>
       </c>
       <c r="I9">
-        <v>1797</v>
+        <v>398</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -10543,26 +10555,26 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
@@ -10588,7 +10600,7 @@
         <v>25</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -10614,10 +10626,10 @@
         <v>350</v>
       </c>
       <c r="H18">
-        <v>2395</v>
+        <v>381</v>
       </c>
       <c r="I18">
-        <v>1710</v>
+        <v>381</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -10643,10 +10655,10 @@
         <v>341</v>
       </c>
       <c r="H19">
-        <v>1734</v>
+        <v>498</v>
       </c>
       <c r="I19">
-        <v>1617</v>
+        <v>366</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -10672,10 +10684,10 @@
         <v>342</v>
       </c>
       <c r="H20">
-        <v>2143</v>
+        <v>423</v>
       </c>
       <c r="I20">
-        <v>933</v>
+        <v>435</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -10701,10 +10713,10 @@
         <v>342</v>
       </c>
       <c r="H21">
-        <v>2735</v>
+        <v>495</v>
       </c>
       <c r="I21">
-        <v>638</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -10730,10 +10742,10 @@
         <v>341</v>
       </c>
       <c r="H22">
-        <v>2283</v>
+        <v>494</v>
       </c>
       <c r="I22">
-        <v>889</v>
+        <v>353</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -10745,26 +10757,26 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
@@ -10790,7 +10802,7 @@
         <v>25</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -10816,10 +10828,10 @@
         <v>341</v>
       </c>
       <c r="H31">
-        <v>472</v>
+        <v>405</v>
       </c>
       <c r="I31">
-        <v>401</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -10845,7 +10857,7 @@
         <v>342</v>
       </c>
       <c r="H32">
-        <v>500</v>
+        <v>386</v>
       </c>
       <c r="I32">
         <v>371</v>
@@ -10874,7 +10886,7 @@
         <v>350</v>
       </c>
       <c r="H33">
-        <v>466</v>
+        <v>527</v>
       </c>
       <c r="I33">
         <v>393</v>
@@ -10903,10 +10915,10 @@
         <v>342</v>
       </c>
       <c r="H34">
-        <v>506</v>
+        <v>430</v>
       </c>
       <c r="I34">
-        <v>390</v>
+        <v>357</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -10932,7 +10944,7 @@
         <v>350</v>
       </c>
       <c r="H35">
-        <v>634</v>
+        <v>388</v>
       </c>
       <c r="I35">
         <v>344</v>
@@ -10947,26 +10959,26 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
+      <c r="A41" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
     </row>
     <row r="43" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
@@ -10992,7 +11004,7 @@
         <v>25</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -11018,10 +11030,10 @@
         <v>341</v>
       </c>
       <c r="H44">
-        <v>2250</v>
+        <v>425</v>
       </c>
       <c r="I44">
-        <v>1508</v>
+        <v>435</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -11047,10 +11059,10 @@
         <v>349</v>
       </c>
       <c r="H45">
-        <v>3093</v>
+        <v>415</v>
       </c>
       <c r="I45">
-        <v>2217</v>
+        <v>332</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -11076,10 +11088,10 @@
         <v>342</v>
       </c>
       <c r="H46">
-        <v>3045</v>
+        <v>393</v>
       </c>
       <c r="I46">
-        <v>1225</v>
+        <v>407</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -11105,10 +11117,10 @@
         <v>341</v>
       </c>
       <c r="H47">
-        <v>1958</v>
+        <v>455</v>
       </c>
       <c r="I47">
-        <v>2303</v>
+        <v>414</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -11134,10 +11146,10 @@
         <v>342</v>
       </c>
       <c r="H48">
-        <v>4265</v>
+        <v>385</v>
       </c>
       <c r="I48">
-        <v>2296</v>
+        <v>362</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -11152,26 +11164,26 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
+      <c r="A54" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="13" t="s">
+      <c r="A55" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="13"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="14"/>
     </row>
     <row r="56" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
@@ -11197,7 +11209,7 @@
         <v>25</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -11223,10 +11235,10 @@
         <v>353</v>
       </c>
       <c r="H57">
-        <v>971</v>
+        <v>536</v>
       </c>
       <c r="I57">
-        <v>1350</v>
+        <v>235</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -11252,10 +11264,10 @@
         <v>341</v>
       </c>
       <c r="H58">
-        <v>2641</v>
+        <v>308</v>
       </c>
       <c r="I58">
-        <v>474</v>
+        <v>349</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -11281,10 +11293,10 @@
         <v>341</v>
       </c>
       <c r="H59">
-        <v>2244</v>
+        <v>293</v>
       </c>
       <c r="I59">
-        <v>697</v>
+        <v>295</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -11310,10 +11322,10 @@
         <v>342</v>
       </c>
       <c r="H60">
-        <v>3137</v>
+        <v>562</v>
       </c>
       <c r="I60">
-        <v>1559</v>
+        <v>324</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -11339,33 +11351,33 @@
         <v>341</v>
       </c>
       <c r="H61">
-        <v>1010</v>
+        <v>326</v>
       </c>
       <c r="I61">
-        <v>1070</v>
+        <v>313</v>
       </c>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16"/>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
+      <c r="A66" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B66" s="13"/>
-      <c r="C66" s="13"/>
-      <c r="D66" s="13"/>
-      <c r="E66" s="13"/>
-      <c r="F66" s="13"/>
-      <c r="G66" s="13"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="14"/>
+      <c r="G66" s="14"/>
     </row>
     <row r="67" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="9"/>
@@ -11391,7 +11403,7 @@
         <v>33</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
@@ -11424,11 +11436,11 @@
       </c>
       <c r="H68">
         <f>AVERAGE(H5:H9)</f>
-        <v>3773.6</v>
+        <v>436.6</v>
       </c>
       <c r="I68">
         <f>AVERAGE(I5:I9)</f>
-        <v>1717.4</v>
+        <v>375.2</v>
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.25">
@@ -11461,11 +11473,11 @@
       </c>
       <c r="H69">
         <f>AVERAGE(H18:H22)</f>
-        <v>2258</v>
+        <v>458.2</v>
       </c>
       <c r="I69">
         <f>AVERAGE(I18:I22)</f>
-        <v>1157.4000000000001</v>
+        <v>388.6</v>
       </c>
       <c r="O69" s="9"/>
       <c r="P69" s="1" t="s">
@@ -11475,10 +11487,10 @@
         <v>0</v>
       </c>
       <c r="R69" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="S69" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.25">
@@ -11511,30 +11523,30 @@
       </c>
       <c r="H70">
         <f>AVERAGE(H31:H35)</f>
-        <v>515.6</v>
+        <v>427.2</v>
       </c>
       <c r="I70">
         <f>AVERAGE(I31:I35)</f>
-        <v>379.8</v>
+        <v>370.6</v>
       </c>
       <c r="O70" s="2">
         <v>0.7</v>
       </c>
-      <c r="P70" s="20">
+      <c r="P70" s="13">
         <f>(G68 - F68) / G68</f>
         <v>-0.12253193960511048</v>
       </c>
-      <c r="Q70" s="20">
+      <c r="Q70" s="13">
         <f>(G68 - G68) / G68</f>
         <v>0</v>
       </c>
-      <c r="R70" s="20">
+      <c r="R70" s="13">
         <f>(G68 - H68) / G68</f>
-        <v>-9.9570267131242733</v>
-      </c>
-      <c r="S70" s="20">
+        <v>-0.26771196283391419</v>
+      </c>
+      <c r="S70" s="13">
         <f>(G68 - I68) / G68</f>
-        <v>-3.9866434378629503</v>
+        <v>-8.9430894308943132E-2</v>
       </c>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.25">
@@ -11567,30 +11579,30 @@
       </c>
       <c r="H71">
         <f>AVERAGE(H44:H48)</f>
-        <v>2922.2</v>
+        <v>414.6</v>
       </c>
       <c r="I71">
         <f>AVERAGE(I44:I48)</f>
-        <v>1909.8</v>
+        <v>390</v>
       </c>
       <c r="O71" s="3">
         <v>0.3</v>
       </c>
-      <c r="P71" s="20">
+      <c r="P71" s="13">
         <f t="shared" ref="P71:P74" si="4">(G69 - F69) / G69</f>
         <v>-0.13403263403263405</v>
       </c>
-      <c r="Q71" s="20">
+      <c r="Q71" s="13">
         <f t="shared" ref="Q71:Q74" si="5">(G69 - G69) / G69</f>
         <v>0</v>
       </c>
-      <c r="R71" s="20">
+      <c r="R71" s="13">
         <f t="shared" ref="R71:R74" si="6">(G69 - H69) / G69</f>
-        <v>-5.5792540792540795</v>
-      </c>
-      <c r="S71" s="20">
-        <f t="shared" ref="S71:S74" si="7">(G69 - I69) / G69</f>
-        <v>-2.3723776223776225</v>
+        <v>-0.33508158508158509</v>
+      </c>
+      <c r="S71" s="13">
+        <f t="shared" ref="S71:S73" si="7">(G69 - I69) / G69</f>
+        <v>-0.13228438228438238</v>
       </c>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
@@ -11623,72 +11635,72 @@
       </c>
       <c r="H72">
         <f>AVERAGE(H57:H61)</f>
-        <v>2000.6</v>
+        <v>405</v>
       </c>
       <c r="I72">
         <f>AVERAGE(I57:I61)</f>
-        <v>1030</v>
+        <v>303.2</v>
       </c>
       <c r="O72" s="3">
         <v>0</v>
       </c>
-      <c r="P72" s="20">
+      <c r="P72" s="13">
         <f t="shared" si="4"/>
         <v>-5.5072463768115941E-2</v>
       </c>
-      <c r="Q72" s="20">
+      <c r="Q72" s="13">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R72" s="20">
+      <c r="R72" s="13">
         <f t="shared" si="6"/>
-        <v>-0.49449275362318845</v>
-      </c>
-      <c r="S72" s="20">
+        <v>-0.23826086956521736</v>
+      </c>
+      <c r="S72" s="13">
         <f t="shared" si="7"/>
-        <v>-0.10086956521739134</v>
+        <v>-7.4202898550724705E-2</v>
       </c>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="O73" s="3">
         <v>-0.3</v>
       </c>
-      <c r="P73" s="20">
+      <c r="P73" s="13">
         <f t="shared" si="4"/>
         <v>-9.9708454810495589E-2</v>
       </c>
-      <c r="Q73" s="20">
+      <c r="Q73" s="13">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R73" s="20">
+      <c r="R73" s="13">
         <f t="shared" si="6"/>
-        <v>-7.5195335276967921</v>
-      </c>
-      <c r="S73" s="20">
+        <v>-0.20874635568513125</v>
+      </c>
+      <c r="S73" s="13">
         <f t="shared" si="7"/>
-        <v>-4.5679300291545184</v>
+        <v>-0.13702623906705538</v>
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="O74" s="3">
         <v>-0.7</v>
       </c>
-      <c r="P74" s="20">
+      <c r="P74" s="13">
         <f t="shared" si="4"/>
         <v>-0.1577415599534342</v>
       </c>
-      <c r="Q74" s="20">
+      <c r="Q74" s="13">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R74" s="20">
+      <c r="R74" s="13">
         <f t="shared" si="6"/>
-        <v>-4.8224679860302677</v>
-      </c>
-      <c r="S74" s="20">
-        <f t="shared" si="7"/>
-        <v>-1.9976717112922</v>
+        <v>-0.17869615832363206</v>
+      </c>
+      <c r="S74" s="13">
+        <f>(G72 - I72) / G72</f>
+        <v>0.11757857974388833</v>
       </c>
     </row>
   </sheetData>
@@ -11728,26 +11740,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
@@ -11773,7 +11785,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -11799,10 +11811,10 @@
         <v>1.46</v>
       </c>
       <c r="H4">
-        <v>5.4820000000000002</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="I4">
-        <v>2.46</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -11828,10 +11840,10 @@
         <v>1.181</v>
       </c>
       <c r="H5">
-        <v>6.1589999999999998</v>
+        <v>3.1440000000000001</v>
       </c>
       <c r="I5">
-        <v>3.5009999999999999</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -11857,10 +11869,10 @@
         <v>1.8640000000000001</v>
       </c>
       <c r="H6">
-        <v>5.484</v>
+        <v>3.0350000000000001</v>
       </c>
       <c r="I6">
-        <v>2.2789999999999999</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -11886,10 +11898,10 @@
         <v>1.099</v>
       </c>
       <c r="H7">
-        <v>5.3630000000000004</v>
+        <v>3.351</v>
       </c>
       <c r="I7">
-        <v>2.1320000000000001</v>
+        <v>3.1320000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -11915,33 +11927,33 @@
         <v>1.032</v>
       </c>
       <c r="H8">
-        <v>5.7750000000000004</v>
+        <v>3.1560000000000001</v>
       </c>
       <c r="I8">
-        <v>2.524</v>
+        <v>3.0150000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="19"/>
     </row>
     <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
@@ -11967,7 +11979,7 @@
         <v>25</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -11993,10 +12005,10 @@
         <v>1.2050000000000001</v>
       </c>
       <c r="H16">
-        <v>4.976</v>
+        <v>2.8679999999999999</v>
       </c>
       <c r="I16">
-        <v>2.2269999999999999</v>
+        <v>2.9380000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -12022,10 +12034,10 @@
         <v>1.419</v>
       </c>
       <c r="H17">
-        <v>4.9320000000000004</v>
+        <v>2.9630000000000001</v>
       </c>
       <c r="I17">
-        <v>2.3010000000000002</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -12051,10 +12063,10 @@
         <v>1.4910000000000001</v>
       </c>
       <c r="H18">
-        <v>5.3620000000000001</v>
+        <v>2.9830000000000001</v>
       </c>
       <c r="I18">
-        <v>2.1890000000000001</v>
+        <v>3.1549999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -12080,10 +12092,10 @@
         <v>1.5129999999999999</v>
       </c>
       <c r="H19">
-        <v>3.9649999999999999</v>
+        <v>2.992</v>
       </c>
       <c r="I19">
-        <v>2.1669999999999998</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -12109,33 +12121,33 @@
         <v>1.4950000000000001</v>
       </c>
       <c r="H20">
-        <v>4.2039999999999997</v>
+        <v>3.226</v>
       </c>
       <c r="I20">
-        <v>2.1349999999999998</v>
+        <v>3.133</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
@@ -12161,7 +12173,7 @@
         <v>25</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -12187,10 +12199,10 @@
         <v>0.93100000000000005</v>
       </c>
       <c r="H27">
-        <v>4.4020000000000001</v>
+        <v>2.8079999999999998</v>
       </c>
       <c r="I27">
-        <v>2.0019999999999998</v>
+        <v>2.8079999999999998</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -12216,10 +12228,10 @@
         <v>0.80700000000000005</v>
       </c>
       <c r="H28">
-        <v>4.9240000000000004</v>
+        <v>3.0259999999999998</v>
       </c>
       <c r="I28">
-        <v>2.157</v>
+        <v>3.0259999999999998</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -12245,10 +12257,10 @@
         <v>1.004</v>
       </c>
       <c r="H29">
-        <v>4.59</v>
+        <v>3.0830000000000002</v>
       </c>
       <c r="I29">
-        <v>1.98</v>
+        <v>3.0830000000000002</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -12274,10 +12286,10 @@
         <v>1.1830000000000001</v>
       </c>
       <c r="H30">
-        <v>4.4969999999999999</v>
+        <v>3.2330000000000001</v>
       </c>
       <c r="I30">
-        <v>2.25</v>
+        <v>3.0329999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -12303,33 +12315,33 @@
         <v>1.2</v>
       </c>
       <c r="H31">
-        <v>4.9409999999999998</v>
+        <v>3.0590000000000002</v>
       </c>
       <c r="I31">
-        <v>1.9510000000000001</v>
+        <v>2.9590000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+      <c r="A36" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="19"/>
     </row>
     <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
@@ -12355,7 +12367,7 @@
         <v>25</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -12381,10 +12393,10 @@
         <v>0.79100000000000004</v>
       </c>
       <c r="H38">
-        <v>5.3090000000000002</v>
+        <v>3.2069999999999999</v>
       </c>
       <c r="I38">
-        <v>2.5499999999999998</v>
+        <v>3.0070000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -12410,10 +12422,10 @@
         <v>1.19</v>
       </c>
       <c r="H39">
-        <v>5.3639999999999999</v>
+        <v>3.0590000000000002</v>
       </c>
       <c r="I39">
-        <v>2.452</v>
+        <v>3.0089999999999999</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -12439,10 +12451,10 @@
         <v>1.0509999999999999</v>
       </c>
       <c r="H40">
-        <v>4.9809999999999999</v>
+        <v>3.0590000000000002</v>
       </c>
       <c r="I40">
-        <v>2.1859999999999999</v>
+        <v>3.0089999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -12468,10 +12480,10 @@
         <v>1.01</v>
       </c>
       <c r="H41">
-        <v>5.343</v>
+        <v>2.9980000000000002</v>
       </c>
       <c r="I41">
-        <v>2.387</v>
+        <v>2.8980000000000001</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -12497,33 +12509,33 @@
         <v>1.113</v>
       </c>
       <c r="H42">
-        <v>4.5629999999999997</v>
+        <v>3.1890000000000001</v>
       </c>
       <c r="I42">
-        <v>2.2389999999999999</v>
+        <v>3.089</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
+      <c r="A47" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
+      <c r="A48" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="19"/>
     </row>
     <row r="49" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
@@ -12549,7 +12561,7 @@
         <v>25</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -12575,7 +12587,7 @@
         <v>0.72599999999999998</v>
       </c>
       <c r="H50">
-        <v>3.7080000000000002</v>
+        <v>3.2989999999999999</v>
       </c>
       <c r="I50">
         <v>2.992</v>
@@ -12698,26 +12710,26 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="13" t="s">
+      <c r="A60" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B60" s="13"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="13"/>
-      <c r="F60" s="13"/>
-      <c r="G60" s="13"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
+      <c r="G60" s="14"/>
     </row>
     <row r="61" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>
@@ -12740,10 +12752,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -12776,11 +12788,11 @@
       </c>
       <c r="H62">
         <f>AVERAGE(H4:H8)</f>
-        <v>5.6525999999999996</v>
+        <v>3.1916000000000002</v>
       </c>
       <c r="I62">
         <f>AVERAGE(I4:I8)</f>
-        <v>2.5792000000000002</v>
+        <v>3.1394000000000002</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -12813,11 +12825,11 @@
       </c>
       <c r="H63">
         <f>AVERAGE(H16:H20)</f>
-        <v>4.6878000000000002</v>
+        <v>3.0064000000000002</v>
       </c>
       <c r="I63">
         <f>AVERAGE(I16:I20)</f>
-        <v>2.2038000000000002</v>
+        <v>3.2231999999999998</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -12850,11 +12862,11 @@
       </c>
       <c r="H64">
         <f>AVERAGE(H27:H31)</f>
-        <v>4.6707999999999998</v>
+        <v>3.0417999999999998</v>
       </c>
       <c r="I64">
         <f>AVERAGE(I27:I31)</f>
-        <v>2.0680000000000001</v>
+        <v>2.9817999999999998</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -12887,11 +12899,11 @@
       </c>
       <c r="H65">
         <f>AVERAGE(H38:H42)</f>
-        <v>5.1120000000000001</v>
+        <v>3.1024000000000003</v>
       </c>
       <c r="I65">
         <f>AVERAGE(I38:I42)</f>
-        <v>2.3628</v>
+        <v>3.0024000000000002</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -12924,7 +12936,7 @@
       </c>
       <c r="H66">
         <f>AVERAGE(H50:H54)</f>
-        <v>4.0469999999999997</v>
+        <v>3.9652000000000003</v>
       </c>
       <c r="I66">
         <f>AVERAGE(I50:I54)</f>
@@ -12966,26 +12978,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
@@ -13011,7 +13023,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -13040,7 +13052,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>2.0879999999999999E-2</v>
+        <v>9.9900000000000003E-2</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -13069,7 +13081,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>2.58E-2</v>
+        <v>9.9900000000000003E-2</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -13098,7 +13110,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>1.9699999999999999E-2</v>
+        <v>0.14799999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -13127,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>2.665E-2</v>
+        <v>9.9900000000000003E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -13156,15 +13168,15 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>2.2599999999999999E-2</v>
+        <v>8.2600000000000007E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
@@ -13194,7 +13206,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="4">
-        <v>1.76685E-2</v>
+        <v>9.5200000000000007E-2</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -13211,7 +13223,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="4">
-        <v>2.6088E-2</v>
+        <v>0.17599999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -13228,7 +13240,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="4">
-        <v>2.0779599999999999E-2</v>
+        <v>0.18240000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -13245,7 +13257,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="4">
-        <v>2.639E-2</v>
+        <v>0.17599999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -13262,31 +13274,31 @@
         <v>0</v>
       </c>
       <c r="E16" s="4">
-        <v>2.5659999999999999E-2</v>
+        <v>0.15565999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
@@ -13312,7 +13324,7 @@
         <v>25</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -13341,7 +13353,7 @@
         <v>0</v>
       </c>
       <c r="I24">
-        <v>2.5499999999999998E-2</v>
+        <v>9.9959999999999993E-2</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -13370,7 +13382,7 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>2.58E-2</v>
+        <v>2.6100000000000002E-2</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -13399,7 +13411,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>3.0099999999999998E-2</v>
+        <v>7.4999999999999997E-2</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -13428,7 +13440,7 @@
         <v>0</v>
       </c>
       <c r="I27">
-        <v>2.4400000000000002E-2</v>
+        <v>9.3899999999999997E-2</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -13457,15 +13469,15 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>1.7420000000000001E-2</v>
+        <v>9.9900000000000003E-2</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
@@ -13495,7 +13507,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="4">
-        <v>2.2290000000000001E-2</v>
+        <v>0.1152</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -13512,7 +13524,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="4">
-        <v>2.2409999999999999E-2</v>
+        <v>2.6669999999999999E-2</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -13529,7 +13541,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="4">
-        <v>2.845E-2</v>
+        <v>7.9829999999999998E-2</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -13546,7 +13558,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="4">
-        <v>2.1590000000000002E-2</v>
+        <v>9.9860000000000004E-2</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -13563,30 +13575,30 @@
         <v>0</v>
       </c>
       <c r="E36" s="4">
-        <v>1.7108999999999999E-2</v>
+        <v>0.12235</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
+      <c r="A40" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
@@ -13612,7 +13624,7 @@
         <v>25</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -13641,7 +13653,7 @@
         <v>0</v>
       </c>
       <c r="I43">
-        <v>3.3799999999999997E-2</v>
+        <v>8.3799999999999999E-2</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -13670,7 +13682,7 @@
         <v>0</v>
       </c>
       <c r="I44">
-        <v>4.3400000000000001E-2</v>
+        <v>7.3400000000000007E-2</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -13699,7 +13711,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3.0110000000000001E-2</v>
+        <v>9.0109999999999996E-2</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -13728,7 +13740,7 @@
         <v>0</v>
       </c>
       <c r="I46">
-        <v>2.69E-2</v>
+        <v>9.69E-2</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -13757,15 +13769,15 @@
         <v>0</v>
       </c>
       <c r="I47">
-        <v>2.537E-2</v>
+        <v>8.5370000000000001E-2</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
@@ -13867,26 +13879,26 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="14" t="s">
+      <c r="A59" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="13" t="s">
+      <c r="A60" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B60" s="13"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="13"/>
-      <c r="F60" s="13"/>
-      <c r="G60" s="13"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
+      <c r="G60" s="14"/>
     </row>
     <row r="61" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="5"/>
@@ -13912,7 +13924,7 @@
         <v>25</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -13941,7 +13953,7 @@
         <v>0</v>
       </c>
       <c r="I62">
-        <v>1.409E-2</v>
+        <v>8.3799999999999999E-2</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -13970,7 +13982,7 @@
         <v>0</v>
       </c>
       <c r="I63">
-        <v>8.0700000000000008E-3</v>
+        <v>8.3400000000000002E-2</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -13999,7 +14011,7 @@
         <v>0</v>
       </c>
       <c r="I64">
-        <v>2.8400000000000002E-2</v>
+        <v>9.0109999999999996E-2</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -14028,7 +14040,7 @@
         <v>0</v>
       </c>
       <c r="I65">
-        <v>2.3400000000000001E-2</v>
+        <v>0.1069</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -14057,15 +14069,15 @@
         <v>0</v>
       </c>
       <c r="I66">
-        <v>4.4699999999999997E-2</v>
+        <v>0.10537000000000001</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" s="19" t="s">
+      <c r="A68" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
+      <c r="B68" s="20"/>
+      <c r="C68" s="20"/>
     </row>
     <row r="69" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B69" s="1" t="s">
@@ -14185,26 +14197,26 @@
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="14" t="s">
+      <c r="A78" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B78" s="14"/>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="15"/>
+      <c r="G78" s="15"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A79" s="13" t="s">
+      <c r="A79" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B79" s="13"/>
-      <c r="C79" s="13"/>
-      <c r="D79" s="13"/>
-      <c r="E79" s="13"/>
-      <c r="F79" s="13"/>
-      <c r="G79" s="13"/>
+      <c r="B79" s="14"/>
+      <c r="C79" s="14"/>
+      <c r="D79" s="14"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="14"/>
+      <c r="G79" s="14"/>
     </row>
     <row r="80" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="5"/>
@@ -14230,7 +14242,7 @@
         <v>25</v>
       </c>
       <c r="I80" s="11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
@@ -14379,11 +14391,11 @@
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="19" t="s">
+      <c r="A87" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B87" s="19"/>
-      <c r="C87" s="19"/>
+      <c r="B87" s="20"/>
+      <c r="C87" s="20"/>
     </row>
     <row r="88" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B88" s="1" t="s">
@@ -14503,26 +14515,26 @@
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" s="15" t="s">
+      <c r="A98" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B98" s="15"/>
-      <c r="C98" s="15"/>
-      <c r="D98" s="15"/>
-      <c r="E98" s="15"/>
-      <c r="F98" s="15"/>
-      <c r="G98" s="15"/>
+      <c r="B98" s="16"/>
+      <c r="C98" s="16"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="16"/>
+      <c r="F98" s="16"/>
+      <c r="G98" s="16"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" s="13" t="s">
+      <c r="A99" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B99" s="13"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="13"/>
-      <c r="E99" s="13"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
+      <c r="B99" s="14"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="14"/>
+      <c r="G99" s="14"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
@@ -14536,60 +14548,60 @@
         <v>0</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F100" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>0.7</v>
       </c>
-      <c r="B101" s="20">
+      <c r="B101" s="13">
         <f>AVERAGE(D4:D8)</f>
         <v>0</v>
       </c>
-      <c r="C101" s="20">
+      <c r="C101" s="13">
         <f>AVERAGE(F4:F8)</f>
         <v>0.48806000000000005</v>
       </c>
-      <c r="D101" s="20">
+      <c r="D101" s="13">
         <f>AVERAGE(G4:G8)</f>
         <v>0.48327999999999999</v>
       </c>
-      <c r="E101" s="20">
+      <c r="E101" s="13">
         <f>AVERAGE(H4:H8)</f>
         <v>0</v>
       </c>
-      <c r="F101" s="20">
+      <c r="F101" s="13">
         <f>AVERAGE(I4:I8)</f>
-        <v>2.3126000000000001E-2</v>
+        <v>0.10606</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>0.3</v>
       </c>
-      <c r="B102" s="20">
+      <c r="B102" s="13">
         <f>AVERAGE(D24:D28)</f>
         <v>0</v>
       </c>
-      <c r="C102" s="20">
+      <c r="C102" s="13">
         <f>AVERAGE(F24:F28)</f>
         <v>0.25796000000000002</v>
       </c>
-      <c r="D102" s="20">
+      <c r="D102" s="13">
         <f>AVERAGE(G24:G28)</f>
         <v>0.28450000000000003</v>
       </c>
-      <c r="E102" s="20">
+      <c r="E102" s="13">
         <f>AVERAGE(H24:H28)</f>
         <v>0</v>
       </c>
-      <c r="F102" s="20">
+      <c r="F102" s="13">
         <f>AVERAGE(I24:I28)</f>
-        <v>2.4644000000000003E-2</v>
+        <v>7.8972000000000001E-2</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
@@ -14600,61 +14612,61 @@
         <f>AVERAGE(D43:D47)</f>
         <v>0</v>
       </c>
-      <c r="C103" s="20">
+      <c r="C103" s="13">
         <f>AVERAGE(F43:F47)</f>
         <v>1.3120000000000001E-2</v>
       </c>
-      <c r="D103" s="20">
+      <c r="D103" s="13">
         <f>AVERAGE(G43:G47)</f>
         <v>8.5600000000000016E-3</v>
       </c>
-      <c r="E103" s="20">
+      <c r="E103" s="13">
         <f>AVERAGE(H43:H47)</f>
         <v>0</v>
       </c>
-      <c r="F103" s="20">
+      <c r="F103" s="13">
         <f>AVERAGE(I43:I47)</f>
-        <v>3.1916E-2</v>
+        <v>8.5916000000000006E-2</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>-0.3</v>
       </c>
-      <c r="B104" s="20">
+      <c r="B104" s="13">
         <f>AVERAGE(D62:D66)</f>
         <v>0.14330000000000001</v>
       </c>
-      <c r="C104" s="20">
+      <c r="C104" s="13">
         <f>AVERAGE(F62:F66)</f>
         <v>0.33940000000000003</v>
       </c>
-      <c r="D104" s="20">
+      <c r="D104" s="13">
         <f>AVERAGE(G62:G66)</f>
         <v>0.34820000000000001</v>
       </c>
-      <c r="E104" s="20">
+      <c r="E104" s="13">
         <f>AVERAGE(H62:H66)</f>
         <v>0</v>
       </c>
-      <c r="F104" s="20">
+      <c r="F104" s="13">
         <f>AVERAGE(I62:I66)</f>
-        <v>2.3731999999999996E-2</v>
+        <v>9.3916000000000013E-2</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>-0.7</v>
       </c>
-      <c r="B105" s="20">
+      <c r="B105" s="13">
         <f>AVERAGE(D81:D85)</f>
         <v>0.42919999999999997</v>
       </c>
-      <c r="C105" s="20">
+      <c r="C105" s="13">
         <f>AVERAGE(F81:F85)</f>
         <v>0.90449999999999997</v>
       </c>
-      <c r="D105" s="20">
+      <c r="D105" s="13">
         <f>AVERAGE(G81:G85)</f>
         <v>0.88205999999999984</v>
       </c>
@@ -14662,20 +14674,20 @@
         <f>AVERAGE(H81:H85)</f>
         <v>0</v>
       </c>
-      <c r="F105" s="20">
+      <c r="F105" s="13">
         <f>AVERAGE(I81:I85)</f>
         <v>1.9438E-2</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E106" s="20"/>
+      <c r="E106" s="13"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" s="19" t="s">
+      <c r="A109" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B109" s="19"/>
-      <c r="C109" s="19"/>
+      <c r="B109" s="20"/>
+      <c r="C109" s="20"/>
     </row>
     <row r="110" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B110" s="1" t="s">
@@ -14691,7 +14703,7 @@
         <v>33</v>
       </c>
       <c r="F110" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
@@ -14714,7 +14726,7 @@
       </c>
       <c r="F111" s="4">
         <f>AVERAGE(E12:E16)</f>
-        <v>2.331722E-2</v>
+        <v>0.157052</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
@@ -14737,7 +14749,7 @@
       </c>
       <c r="F112" s="4">
         <f>AVERAGE(E32:E36)</f>
-        <v>2.2369800000000002E-2</v>
+        <v>8.8782E-2</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -14851,26 +14863,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
@@ -15045,26 +15057,26 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="19"/>
     </row>
     <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
@@ -15239,26 +15251,26 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
@@ -15433,26 +15445,26 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="19"/>
     </row>
     <row r="38" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
@@ -15627,26 +15639,26 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
+      <c r="A48" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
+      <c r="A49" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="19"/>
     </row>
     <row r="50" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
@@ -15821,26 +15833,26 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
+      <c r="A60" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="17"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="19"/>
     </row>
     <row r="61" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>

</xml_diff>